<commit_message>
Add docker-compose down step; update DB header
Add a new section to README explaining how to stop and remove Docker containers with `docker-compose down` (includes command and brief note). Update database.sql header to note a logical PostgreSQL backup. Also update the testing credentials spreadsheet (credenciales_testing.xlsx).
</commit_message>
<xml_diff>
--- a/credenciales_testing.xlsx
+++ b/credenciales_testing.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Clients_System\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{18AEC20C-71F9-4A35-9F3E-6952AADFB2D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D9F05C0-1C95-462E-89B5-5E0E3ABAE782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Administradores" sheetId="1" r:id="rId1"/>
     <sheet name="Clientes" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -29,9 +28,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="19">
   <si>
-    <t>Credenciales - Administradores</t>
-  </si>
-  <si>
     <t>correo</t>
   </si>
   <si>
@@ -62,9 +58,6 @@
     <t>sofia_mendoza</t>
   </si>
   <si>
-    <t>Credenciales - Clientes</t>
-  </si>
-  <si>
     <t>technovation@empresa.com</t>
   </si>
   <si>
@@ -84,6 +77,12 @@
   </si>
   <si>
     <t>grupoorion_user</t>
+  </si>
+  <si>
+    <t>Credenciales Public - Clientes</t>
+  </si>
+  <si>
+    <t>Credenciales Dashboard - Administradores</t>
   </si>
 </sst>
 </file>
@@ -374,53 +373,53 @@
   <sheetData>
     <row r="1" spans="1:3" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
     </row>
     <row r="3" spans="1:3" ht="12" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="C5" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="C6" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -446,53 +445,53 @@
   <sheetData>
     <row r="1" spans="1:3" ht="14.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
     </row>
     <row r="3" spans="1:3" ht="12" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>